<commit_message>
Map card names and angles to the ISB and ISNCSCI standards
So data can move between the verifier, Blender and other software
(OpenSim, motion capture, clinical records) without being misread.

- Card library: new ISB_term column giving each row's motion in ISB
  joint-angle terms (Wu et al. 2005 / 2002), plus Field Definitions rows.
- docs/conventions.md: axis mapping, joint names, ISB signs, the
  shoulder's rotation order, and the ISNCSCI profile naming.
- accesspath/isb.py: verifier <-> ISB frame conversion and ISB
  shoulder plane-of-elevation / elevation from an arm direction.
- data/isncsci.json + accesspath/isncsci.py: ISNCSCI levels, key
  muscles and AIS grades; SCI profiles must be named SCI_<level>_AIS_<grade>
  and check-cards rejects malformed ones. No SCI joint limits yet.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UEvCJX2bMQCcooJE7fGgnQ
</commit_message>
<xml_diff>
--- a/data/card_library.xlsx
+++ b/data/card_library.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profiles" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Population Caps" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Definitions" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Changes From Original" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Cards" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Profiles" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Population Caps" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Field Definitions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Changes From Original" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P37"/>
+  <dimension ref="A1:Q37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -473,6 +473,7 @@
     <col width="50" customWidth="1" min="14" max="14"/>
     <col width="40" customWidth="1" min="15" max="15"/>
     <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="55" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -556,6 +557,11 @@
           <t>status</t>
         </is>
       </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>ISB_term</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -626,6 +632,11 @@
           <t>sourced</t>
         </is>
       </c>
+      <c r="Q2" s="3" t="inlineStr">
+        <is>
+          <t>Thoracohumeral elevation in plane of elevation 90° (forward); Y-X-Y; Wu et al. 2005 (ISB Part II) 2.4.7</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -698,6 +709,11 @@
       <c r="P3" s="4" t="inlineStr">
         <is>
           <t>interpolated</t>
+        </is>
+      </c>
+      <c r="Q3" s="4" t="inlineStr">
+        <is>
+          <t>Thoracohumeral elevation behind the body (plane of elevation about -90°); Y-X-Y; Wu et al. 2005 (ISB Part II) 2.4.7</t>
         </is>
       </c>
     </row>
@@ -770,6 +786,11 @@
           <t>sourced</t>
         </is>
       </c>
+      <c r="Q4" s="3" t="inlineStr">
+        <is>
+          <t>Thoracohumeral elevation in plane of elevation 0° (sideways); Y-X-Y; Wu et al. 2005 (ISB Part II) 2.4.7</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -840,6 +861,11 @@
           <t>sourced</t>
         </is>
       </c>
+      <c r="Q5" s="3" t="inlineStr">
+        <is>
+          <t>Elbow flexion, +α about humerus Z; Z-X-Y; Wu et al. 2005 (ISB Part II) 3.4.1</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -910,6 +936,11 @@
           <t>sourced</t>
         </is>
       </c>
+      <c r="Q6" s="3" t="inlineStr">
+        <is>
+          <t>Radiocarpal flexion, +α about radius Z; Wu et al. 2005 (ISB Part II) 4.4.1</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -980,6 +1011,11 @@
           <t>sourced</t>
         </is>
       </c>
+      <c r="Q7" s="3" t="inlineStr">
+        <is>
+          <t>Radiocarpal extension, -α about radius Z; Wu et al. 2005 (ISB Part II) 4.4.1</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1050,6 +1086,11 @@
           <t>sourced</t>
         </is>
       </c>
+      <c r="Q8" s="3" t="inlineStr">
+        <is>
+          <t>Hip flexion, +α about pelvis Z; Wu et al. 2002 (ISB Part I)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1120,6 +1161,11 @@
           <t>sourced</t>
         </is>
       </c>
+      <c r="Q9" s="3" t="inlineStr">
+        <is>
+          <t>Knee flexion; Grood &amp; Suntay 1983 (the knee convention ISB uses)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1190,6 +1236,11 @@
           <t>sourced</t>
         </is>
       </c>
+      <c r="Q10" s="3" t="inlineStr">
+        <is>
+          <t>Ankle dorsiflexion, +α; Wu et al. 2002 (ISB Part I)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1260,6 +1311,11 @@
           <t>sourced</t>
         </is>
       </c>
+      <c r="Q11" s="3" t="inlineStr">
+        <is>
+          <t>Ankle plantarflexion, -α; Wu et al. 2002 (ISB Part I)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1330,6 +1386,11 @@
           <t>sourced</t>
         </is>
       </c>
+      <c r="Q12" s="3" t="inlineStr">
+        <is>
+          <t>Thoracohumeral elevation in plane of elevation 90° (forward); Y-X-Y; Wu et al. 2005 (ISB Part II) 2.4.7</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1402,6 +1463,11 @@
       <c r="P13" s="4" t="inlineStr">
         <is>
           <t>interpolated</t>
+        </is>
+      </c>
+      <c r="Q13" s="4" t="inlineStr">
+        <is>
+          <t>Thoracohumeral elevation behind the body (plane of elevation about -90°); Y-X-Y; Wu et al. 2005 (ISB Part II) 2.4.7</t>
         </is>
       </c>
     </row>
@@ -1474,6 +1540,11 @@
           <t>sourced</t>
         </is>
       </c>
+      <c r="Q14" s="3" t="inlineStr">
+        <is>
+          <t>Thoracohumeral elevation in plane of elevation 0° (sideways); Y-X-Y; Wu et al. 2005 (ISB Part II) 2.4.7</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1544,6 +1615,11 @@
           <t>sourced</t>
         </is>
       </c>
+      <c r="Q15" s="3" t="inlineStr">
+        <is>
+          <t>Elbow flexion, +α about humerus Z; Z-X-Y; Wu et al. 2005 (ISB Part II) 3.4.1</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1614,6 +1690,11 @@
           <t>sourced</t>
         </is>
       </c>
+      <c r="Q16" s="3" t="inlineStr">
+        <is>
+          <t>Radiocarpal flexion, +α about radius Z; Wu et al. 2005 (ISB Part II) 4.4.1</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1684,6 +1765,11 @@
           <t>sourced</t>
         </is>
       </c>
+      <c r="Q17" s="3" t="inlineStr">
+        <is>
+          <t>Radiocarpal extension, -α about radius Z; Wu et al. 2005 (ISB Part II) 4.4.1</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1754,6 +1840,11 @@
           <t>sourced</t>
         </is>
       </c>
+      <c r="Q18" s="3" t="inlineStr">
+        <is>
+          <t>Hip flexion, +α about pelvis Z; Wu et al. 2002 (ISB Part I)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1824,6 +1915,11 @@
           <t>sourced</t>
         </is>
       </c>
+      <c r="Q19" s="3" t="inlineStr">
+        <is>
+          <t>Knee flexion; Grood &amp; Suntay 1983 (the knee convention ISB uses)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1894,6 +1990,11 @@
           <t>sourced</t>
         </is>
       </c>
+      <c r="Q20" s="3" t="inlineStr">
+        <is>
+          <t>Ankle dorsiflexion, +α; Wu et al. 2002 (ISB Part I)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1964,6 +2065,11 @@
           <t>sourced</t>
         </is>
       </c>
+      <c r="Q21" s="3" t="inlineStr">
+        <is>
+          <t>Ankle plantarflexion, -α; Wu et al. 2002 (ISB Part I)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2038,6 +2144,11 @@
           <t>interpolated</t>
         </is>
       </c>
+      <c r="Q22" s="4" t="inlineStr">
+        <is>
+          <t>Thorax flexion relative to pelvis (Wu et al. 2002 (ISB Part I)); Wu et al. 2005 (ISB Part II) 2.4.1 gives thorax vs. global, flexion = -α about Z</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -2112,6 +2223,11 @@
           <t>sourced</t>
         </is>
       </c>
+      <c r="Q23" s="3" t="inlineStr">
+        <is>
+          <t>Thoracohumeral elevation in plane of elevation 0° (sideways); Y-X-Y; Wu et al. 2005 (ISB Part II) 2.4.7</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2186,6 +2302,11 @@
           <t>sourced</t>
         </is>
       </c>
+      <c r="Q24" s="3" t="inlineStr">
+        <is>
+          <t>Thoracohumeral elevation in plane of elevation 0° (sideways); Y-X-Y; Wu et al. 2005 (ISB Part II) 2.4.7</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2260,6 +2381,11 @@
           <t>sourced</t>
         </is>
       </c>
+      <c r="Q25" s="3" t="inlineStr">
+        <is>
+          <t>Thoracohumeral elevation in plane of elevation 0° (sideways); Y-X-Y; Wu et al. 2005 (ISB Part II) 2.4.7</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2332,6 +2458,11 @@
       <c r="P26" s="3" t="inlineStr">
         <is>
           <t>sourced</t>
+        </is>
+      </c>
+      <c r="Q26" s="3" t="inlineStr">
+        <is>
+          <t>Thoracohumeral elevation in plane of elevation 0° (sideways); Y-X-Y; Wu et al. 2005 (ISB Part II) 2.4.7</t>
         </is>
       </c>
     </row>
@@ -2406,6 +2537,11 @@
           <t>sourced</t>
         </is>
       </c>
+      <c r="Q27" s="3" t="inlineStr">
+        <is>
+          <t>Thoracohumeral elevation in plane of elevation 90° (forward); Y-X-Y; Wu et al. 2005 (ISB Part II) 2.4.7</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2478,6 +2614,11 @@
           <t>sourced</t>
         </is>
       </c>
+      <c r="Q28" s="3" t="inlineStr">
+        <is>
+          <t>Elbow flexion, +α about humerus Z; Z-X-Y; Wu et al. 2005 (ISB Part II) 3.4.1</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2554,6 +2695,11 @@
       <c r="P29" s="4" t="inlineStr">
         <is>
           <t>interpolated</t>
+        </is>
+      </c>
+      <c r="Q29" s="4" t="inlineStr">
+        <is>
+          <t>Knee flexion; Grood &amp; Suntay 1983 (the knee convention ISB uses)</t>
         </is>
       </c>
     </row>
@@ -2618,6 +2764,11 @@
           <t>placeholder</t>
         </is>
       </c>
+      <c r="Q30" s="5" t="inlineStr">
+        <is>
+          <t>n/a: functional measure, not a joint angle</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2680,6 +2831,11 @@
           <t>placeholder</t>
         </is>
       </c>
+      <c r="Q31" s="5" t="inlineStr">
+        <is>
+          <t>Thoracohumeral elevation in plane of elevation 90° (forward); Y-X-Y; Wu et al. 2005 (ISB Part II) 2.4.7</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2742,6 +2898,11 @@
           <t>placeholder</t>
         </is>
       </c>
+      <c r="Q32" s="5" t="inlineStr">
+        <is>
+          <t>Thoracohumeral elevation in plane of elevation 0° (sideways); Y-X-Y; Wu et al. 2005 (ISB Part II) 2.4.7</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2804,6 +2965,11 @@
           <t>placeholder</t>
         </is>
       </c>
+      <c r="Q33" s="5" t="inlineStr">
+        <is>
+          <t>Hip flexion, +α about pelvis Z; Wu et al. 2002 (ISB Part I)</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2866,6 +3032,11 @@
           <t>placeholder</t>
         </is>
       </c>
+      <c r="Q34" s="5" t="inlineStr">
+        <is>
+          <t>Knee flexion; Grood &amp; Suntay 1983 (the knee convention ISB uses)</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2928,6 +3099,11 @@
           <t>placeholder</t>
         </is>
       </c>
+      <c r="Q35" s="5" t="inlineStr">
+        <is>
+          <t>MCP/IP flexion, +α about proximal segment Z; Wu et al. 2005 (ISB Part II) 4.4.1</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2990,6 +3166,11 @@
           <t>placeholder</t>
         </is>
       </c>
+      <c r="Q36" s="5" t="inlineStr">
+        <is>
+          <t>n/a: functional measure, not a joint angle</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -3054,6 +3235,11 @@
       <c r="P37" s="5" t="inlineStr">
         <is>
           <t>placeholder</t>
+        </is>
+      </c>
+      <c r="Q37" s="5" t="inlineStr">
+        <is>
+          <t>n/a: functional measure, not a joint angle</t>
         </is>
       </c>
     </row>
@@ -3529,7 +3715,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B25"/>
+  <dimension ref="A1:B27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3737,76 +3923,100 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr"/>
-      <c r="B18" s="2" t="inlineStr"/>
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>ISB_term</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>The same motion in the International Society of Biomechanics (ISB) joint-angle standard: which ISB angle it is, the rotation order, and the section of the paper. Lets the card be read the same way by other software (OpenSim, motion capture). Numbers stay as degrees from neutral, always positive; ISB signs are in docs/conventions.md.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Profiles sheet</t>
-        </is>
-      </c>
+      <c r="A19" s="2" t="inlineStr"/>
       <c r="B19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>posture</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>standing or seated_wheelchair.</t>
-        </is>
-      </c>
+          <t>Profiles sheet</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>mobility_aid</t>
+          <t>posture</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>none, wheelchair, crutches, KAFO. Used for doorway clearance.</t>
+          <t>standing or seated_wheelchair.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>affected_side</t>
+          <t>mobility_aid</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>R, L, both, or none. Decides which side '_affected' cards apply to.</t>
+          <t>none, wheelchair, crutches, KAFO. Used for doorway clearance.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
+          <t>affected_side</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>R, L, both, or none. Decides which side '_affected' cards apply to.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
           <t>card_ids</t>
         </is>
       </c>
-      <c r="B23" s="2" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>Comma-separated card_ids from the Cards sheet. Baseline cards are always applied first.</t>
         </is>
       </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr"/>
-      <c r="B24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
+          <t>profile_id</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Any name. Spinal cord injury profiles must be named the ISNCSCI way, SCI_&lt;level&gt;_AIS_&lt;grade&gt; (e.g. SCI_C6_AIS_A), optionally with _wheelchair etc. after it; check-cards rejects a malformed SCI_ name.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr"/>
+      <c r="B26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
           <t>Population Caps sheet</t>
         </is>
       </c>
-      <c r="B25" s="2" t="inlineStr">
+      <c r="B27" s="2" t="inlineStr">
         <is>
           <t>Population-level statistics that are not a per-joint limit. Shown as a CAUTION on matching results.</t>
         </is>
@@ -3823,7 +4033,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -3920,6 +4130,13 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Added ISB_term: each row's motion in ISB joint-angle terms, so the library can move between software.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add body-size bands and a dial within each card's range
- Body Bands sheet: four 4-inch height ranges (A to D) covering the 5th
  to 95th percentile of U.S. adults (CDC NHANES 2015-2018, Tables 10
  and 12). Reach is tested at a band's shortest height; a measured
  height within the band can be dialled in instead.
- Profiles can dial a card to a value inside its range with
  card_id@value (e.g. stroke-shoulder-abd-1@60). Blank keeps the
  cautious edge; out-of-range values and placeholders are rejected.
- load_body takes a height; each result records which body was tested.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UEvCJX2bMQCcooJE7fGgnQ
</commit_message>
<xml_diff>
--- a/data/card_library.xlsx
+++ b/data/card_library.xlsx
@@ -10,8 +10,9 @@
     <sheet name="Cards" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Profiles" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Population Caps" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Field Definitions" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Changes From Original" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Body Bands" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Field Definitions" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Changes From Original" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3254,7 +3255,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3294,6 +3295,16 @@
       <c r="F1" s="1" t="inlineStr">
         <is>
           <t>card_ids</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>body_band</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>body_height_in</t>
         </is>
       </c>
     </row>
@@ -3715,310 +3726,184 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B27"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="100" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="70" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Field</t>
+          <t>band_id</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Holds</t>
+          <t>label</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>stature_min_in</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>stature_max_in</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>status</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Cards sheet</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr"/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>4 ft 11 in to 5 ft 3 in</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>59</v>
+      </c>
+      <c r="D2" t="n">
+        <v>63</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>4-inch band. Reach is tested at the shortest height, room (knees, head, doors) at the tallest. Band edges are a design choice anchored to the CDC percentiles.</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>CDC/NCHS, Anthropometric Reference Data for Children and Adults: United States, 2015-2018 (Fryar et al., Vital Health Stat 3(46), 2021), Tables 10 and 12: adult women 5th percentile 59.0 in, adult men 95th percentile 73.8 in</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>interpolated</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>card_id</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Unique name for the row. Profiles list the card_ids they use, so editing a row updates every profile that uses it.</t>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>5 ft 3 in to 5 ft 7 in</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>63</v>
+      </c>
+      <c r="D3" t="n">
+        <v>67</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>4-inch band. Reach is tested at the shortest height, room (knees, head, doors) at the tallest. Band edges are a design choice anchored to the CDC percentiles.</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>CDC/NCHS, Anthropometric Reference Data for Children and Adults: United States, 2015-2018 (Fryar et al., Vital Health Stat 3(46), 2021), Tables 10 and 12: adult women 5th percentile 59.0 in, adult men 95th percentile 73.8 in</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>interpolated</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>joint_id</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>shoulder_R, knee_L, trunk ... Condition rows use '_affected': the profile's affected_side decides which side(s) that means.</t>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>5 ft 7 in to 5 ft 11 in</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>67</v>
+      </c>
+      <c r="D4" t="n">
+        <v>71</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>4-inch band. Reach is tested at the shortest height, room (knees, head, doors) at the tallest. Band edges are a design choice anchored to the CDC percentiles.</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>CDC/NCHS, Anthropometric Reference Data for Children and Adults: United States, 2015-2018 (Fryar et al., Vital Health Stat 3(46), 2021), Tables 10 and 12: adult women 5th percentile 59.0 in, adult men 95th percentile 73.8 in</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>interpolated</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>parent_joint</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>What it's chained to in the kinematic chain (elbow's parent = shoulder).</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>DOF_axis</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>One direction of motion per row: flexion, extension, abduction, adduction, dorsiflexion, plantarflexion, or a named functional measure.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>condition</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>'baseline' for the able-bodied control avatar, or a named condition (stroke, hemiplegia, arthritis, KAFO, ...).</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>severity</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Severity/stage tag when the source reports one; 'able-bodied' for baseline rows.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>ROM_min_deg / ROM_max_deg</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Degrees from neutral, always positive. Leave EMPTY (not a dash) when not sourced.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>range_kind</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>How the verifier uses the numbers. joint_limits: the joint can move from 0 to ROM_max. score_band: a clinical scoring band; the verifier uses the band's lower edge so the design has to work for everyone in the band. task_threshold: the angle a task needed; reported, never applied as a limit. sweep_width / envelope_shift / reach_reduction: functional measures, not yet used by the verifier.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>strength</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Weight-bearing / push / pull capacity. Categorical is fine where no numeric source exists.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>control</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Speed and steadiness, kept separate from ROM so tremor/spasticity/ataxia aren't forced into a pure angle limit.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>laterality</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>independent L/R, affected side, either or both sides, or midline.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>dependency_flags</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>How this card restricts another at the same time, e.g. 'requires free hand for balance'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>notes</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>Context a raw number doesn't carry.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>source</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Citation. 'NEEDED: not yet sourced' marks an open gap rather than inventing a number.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>status</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>sourced / interpolated / placeholder. Placeholder rows have empty numbers; the verifier marks any result that depends on them UNVERIFIED.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>ISB_term</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>The same motion in the International Society of Biomechanics (ISB) joint-angle standard: which ISB angle it is, the rotation order, and the section of the paper. Lets the card be read the same way by other software (OpenSim, motion capture). Numbers stay as degrees from neutral, always positive; ISB signs are in docs/conventions.md.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr"/>
-      <c r="B19" s="2" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Profiles sheet</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>posture</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>standing or seated_wheelchair.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>mobility_aid</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>none, wheelchair, crutches, KAFO. Used for doorway clearance.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>affected_side</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>R, L, both, or none. Decides which side '_affected' cards apply to.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>card_ids</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>Comma-separated card_ids from the Cards sheet. Baseline cards are always applied first.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>profile_id</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>Any name. Spinal cord injury profiles must be named the ISNCSCI way, SCI_&lt;level&gt;_AIS_&lt;grade&gt; (e.g. SCI_C6_AIS_A), optionally with _wheelchair etc. after it; check-cards rejects a malformed SCI_ name.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr"/>
-      <c r="B26" s="2" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>Population Caps sheet</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>Population-level statistics that are not a per-joint limit. Shown as a CAUTION on matching results.</t>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>5 ft 11 in to 6 ft 3 in</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>71</v>
+      </c>
+      <c r="D5" t="n">
+        <v>75</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>4-inch band. Reach is tested at the shortest height, room (knees, head, doors) at the tallest. Band edges are a design choice anchored to the CDC percentiles.</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>CDC/NCHS, Anthropometric Reference Data for Children and Adults: United States, 2015-2018 (Fryar et al., Vital Health Stat 3(46), 2021), Tables 10 and 12: adult women 5th percentile 59.0 in, adult men 95th percentile 73.8 in</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>interpolated</t>
         </is>
       </c>
     </row>
@@ -4033,7 +3918,374 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A14"/>
+  <dimension ref="A1:B32"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="100" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Holds</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Cards sheet</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>card_id</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Unique name for the row. Profiles list the card_ids they use, so editing a row updates every profile that uses it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>joint_id</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>shoulder_R, knee_L, trunk ... Condition rows use '_affected': the profile's affected_side decides which side(s) that means.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>parent_joint</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>What it's chained to in the kinematic chain (elbow's parent = shoulder).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>DOF_axis</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>One direction of motion per row: flexion, extension, abduction, adduction, dorsiflexion, plantarflexion, or a named functional measure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>condition</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>'baseline' for the able-bodied control avatar, or a named condition (stroke, hemiplegia, arthritis, KAFO, ...).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>severity</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Severity/stage tag when the source reports one; 'able-bodied' for baseline rows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>ROM_min_deg / ROM_max_deg</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Degrees from neutral, always positive. Leave EMPTY (not a dash) when not sourced.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>range_kind</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>How the verifier uses the numbers. joint_limits: the joint can move from 0 to ROM_max. score_band: a clinical scoring band; the verifier uses the band's lower edge so the design has to work for everyone in the band. task_threshold: the angle a task needed; reported, never applied as a limit. sweep_width / envelope_shift / reach_reduction: functional measures, not yet used by the verifier.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>strength</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Weight-bearing / push / pull capacity. Categorical is fine where no numeric source exists.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Speed and steadiness, kept separate from ROM so tremor/spasticity/ataxia aren't forced into a pure angle limit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>laterality</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>independent L/R, affected side, either or both sides, or midline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>dependency_flags</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>How this card restricts another at the same time, e.g. 'requires free hand for balance'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Context a raw number doesn't carry.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Citation. 'NEEDED: not yet sourced' marks an open gap rather than inventing a number.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>sourced / interpolated / placeholder. Placeholder rows have empty numbers; the verifier marks any result that depends on them UNVERIFIED.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>ISB_term</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>The same motion in the International Society of Biomechanics (ISB) joint-angle standard: which ISB angle it is, the rotation order, and the section of the paper. Lets the card be read the same way by other software (OpenSim, motion capture). Numbers stay as degrees from neutral, always positive; ISB signs are in docs/conventions.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr"/>
+      <c r="B19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Profiles sheet</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>posture</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>standing or seated_wheelchair.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>mobility_aid</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>none, wheelchair, crutches, KAFO. Used for doorway clearance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>affected_side</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>R, L, both, or none. Decides which side '_affected' cards apply to.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>card_ids</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Comma-separated card_ids from the Cards sheet. Baseline cards are always applied first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>card_ids: dial setting</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Optional: write card_id@value to dial a card to a value inside its range, e.g. stroke-shoulder-abd-1@60 (its band is 45 to 90). With no @value the cautious edge is used: a score band's lower edge, a joint limit's max. A value outside the range is rejected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>body_band</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Optional: A, B, C or D from the Body Bands sheet. Blank = the default 1.70 m body in body.json.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>body_height_in</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Optional: a measured height in inches. With a body_band it must fall inside that band; it replaces the band's shortest-height default.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>profile_id</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Any name. Spinal cord injury profiles must be named the ISNCSCI way, SCI_&lt;level&gt;_AIS_&lt;grade&gt; (e.g. SCI_C6_AIS_A), optionally with _wheelchair etc. after it; check-cards rejects a malformed SCI_ name.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr"/>
+      <c r="B29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Population Caps sheet</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Population-level statistics that are not a per-joint limit. Shown as a CAUTION on matching results.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31"/>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Body Bands sheet</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Height ranges treated as one group (4 inches each, covering the 5th to 95th percentile of U.S. adults). Reach is tested at a band's shortest height and room at its tallest. A measured height always beats a band.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -4137,6 +4389,13 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Added Body Bands (4-inch height ranges) and a dial: profiles can set a card or a height to a value inside its range; blank uses the cautious edge.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add two stroke active arm-lift cards (Taketomi 2023, Yim & Kim 2024)
Bands are each study's mean ± 1 SD; the verifier uses the lower edge.
Not used by any profile yet, so results are unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UEvCJX2bMQCcooJE7fGgnQ
</commit_message>
<xml_diff>
--- a/data/card_library.xlsx
+++ b/data/card_library.xlsx
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q37"/>
+  <dimension ref="A1:Q39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2470,7 +2470,7 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>hemi-shoulder-flex-mild</t>
+          <t>stroke-shoulder-flex-weak</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -2490,31 +2490,33 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>hemiplegia</t>
+          <t>stroke</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>mild</t>
-        </is>
-      </c>
-      <c r="G27" s="2" t="n"/>
+          <t>weaker arm (shoulder MMT 2 or less, 6+ months after)</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="n">
+        <v>48.4</v>
+      </c>
       <c r="H27" s="2" t="n">
-        <v>55</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>task_threshold</t>
+          <t>score_band</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>task-dependent</t>
+          <t>reduced</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>reduced</t>
+          <t>variable</t>
         </is>
       </c>
       <c r="L27" s="2" t="inlineStr">
@@ -2525,12 +2527,12 @@
       <c r="M27" s="2" t="n"/>
       <c r="N27" s="2" t="inlineStr">
         <is>
-          <t>Angle needed to complete the reach-behind-head task, not a full ROM max. Not applied as a joint limit.</t>
+          <t>Active lift: how far the person raises the arm forward on their own. Band is the study mean 60.0 ± 1 SD 11.6 degrees (passive, lifted by someone else: 106.3 ± 18.7). Verifier uses the lower edge. Small study (8 people), pre-treatment values. Not in any profile yet.</t>
         </is>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>PMC11115294 (hemiplegia reach-behind-head study)</t>
+          <t>Taketomi et al. 2023, J Clin Med 12(3):1215, doi:10.3390/jcm12031215, results 3.2.1 pre-intervention (PMID 36769862, PMC9917525)</t>
         </is>
       </c>
       <c r="P27" s="3" t="inlineStr">
@@ -2547,17 +2549,17 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>hemi-elbow-flex-mild</t>
+          <t>stroke-shoulder-flex-milder</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>elbow_affected</t>
+          <t>shoulder_affected</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>shoulder_affected</t>
+          <t>trunk</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -2567,31 +2569,33 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>hemiplegia</t>
+          <t>stroke</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>mild</t>
-        </is>
-      </c>
-      <c r="G28" s="2" t="n"/>
+          <t>milder arm (painful, partly dislocated shoulder, 6+ months after)</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="n">
+        <v>116.4</v>
+      </c>
       <c r="H28" s="2" t="n">
-        <v>145</v>
+        <v>137.8</v>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>task_threshold</t>
+          <t>score_band</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>task-dependent</t>
+          <t>reduced</t>
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>reduced</t>
+          <t>mild spasticity (MAS under 1+)</t>
         </is>
       </c>
       <c r="L28" s="2" t="inlineStr">
@@ -2602,12 +2606,12 @@
       <c r="M28" s="2" t="n"/>
       <c r="N28" s="2" t="inlineStr">
         <is>
-          <t>Angle needed to complete the reach-behind-head task, not a full ROM max. Not applied as a joint limit.</t>
+          <t>Active lift, measured standing. Band is the mean of both groups before treatment, 127.1 ± 1 SD 10.7 degrees (groups: 126.48 ± 10.02, n 18; 127.78 ± 11.63, n 17). Verifier uses the lower edge. Ages 50-70. Not in any profile yet.</t>
         </is>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>PMC11115294 (hemiplegia reach-behind-head study)</t>
+          <t>Yim &amp; Kim 2024, Med Sci Monit 30:e944222, doi:10.12659/MSM.944222, Table 2 pre-intervention (PMID 38820090, PMC11149471)</t>
         </is>
       </c>
       <c r="P28" s="3" t="inlineStr">
@@ -2617,24 +2621,24 @@
       </c>
       <c r="Q28" s="3" t="inlineStr">
         <is>
-          <t>Elbow flexion, +α about humerus Z; Z-X-Y; Wu et al. 2005 (ISB Part II) 3.4.1</t>
+          <t>Thoracohumeral elevation in plane of elevation 90° (forward); Y-X-Y; Wu et al. 2005 (ISB Part II) 2.4.7</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>kafo-knee-flex-locked</t>
+          <t>hemi-shoulder-flex-mild</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>knee_affected</t>
+          <t>shoulder_affected</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>hip_affected</t>
+          <t>trunk</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -2644,33 +2648,31 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>KAFO (locked)</t>
+          <t>hemiplegia</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>typical</t>
-        </is>
-      </c>
-      <c r="G29" s="2" t="n">
-        <v>0</v>
-      </c>
+          <t>mild</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="n"/>
       <c r="H29" s="2" t="n">
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>joint_limits</t>
+          <t>task_threshold</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>n/a (mechanically fixed)</t>
+          <t>task-dependent</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>fixed</t>
+          <t>reduced</t>
         </is>
       </c>
       <c r="L29" s="2" t="inlineStr">
@@ -2678,72 +2680,78 @@
           <t>affected side</t>
         </is>
       </c>
-      <c r="M29" s="2" t="inlineStr">
-        <is>
-          <t>requires circumduction or hip-hike to clear the leg</t>
-        </is>
-      </c>
+      <c r="M29" s="2" t="n"/>
       <c r="N29" s="2" t="inlineStr">
         <is>
-          <t>Leg cannot bend. Wearer compensates via circumduction (lateral hip swing) or hip-hike, which this row does not capture.</t>
+          <t>Angle needed to complete the reach-behind-head task, not a full ROM max. Not applied as a joint limit.</t>
         </is>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>General orthotics principle (KAFO knee joint typically locked near full extension); not a specific citation</t>
-        </is>
-      </c>
-      <c r="P29" s="4" t="inlineStr">
-        <is>
-          <t>interpolated</t>
-        </is>
-      </c>
-      <c r="Q29" s="4" t="inlineStr">
-        <is>
-          <t>Knee flexion; Grood &amp; Suntay 1983 (the knee convention ISB uses)</t>
+          <t>PMC11115294 (hemiplegia reach-behind-head study)</t>
+        </is>
+      </c>
+      <c r="P29" s="3" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="Q29" s="3" t="inlineStr">
+        <is>
+          <t>Thoracohumeral elevation in plane of elevation 90° (forward); Y-X-Y; Wu et al. 2005 (ISB Part II) 2.4.7</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>kafo-knee-circumduction</t>
+          <t>hemi-elbow-flex-mild</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>knee_affected</t>
+          <t>elbow_affected</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>hip_affected</t>
+          <t>shoulder_affected</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>lateral sweep (circumduction)</t>
+          <t>flexion</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>KAFO (locked)</t>
+          <t>hemiplegia</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>typical</t>
+          <t>mild</t>
         </is>
       </c>
       <c r="G30" s="2" t="n"/>
-      <c r="H30" s="2" t="n"/>
+      <c r="H30" s="2" t="n">
+        <v>145</v>
+      </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>sweep_width</t>
-        </is>
-      </c>
-      <c r="J30" s="2" t="n"/>
-      <c r="K30" s="2" t="n"/>
+          <t>task_threshold</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>task-dependent</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>reduced</t>
+        </is>
+      </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
           <t>affected side</t>
@@ -2752,39 +2760,39 @@
       <c r="M30" s="2" t="n"/>
       <c r="N30" s="2" t="inlineStr">
         <is>
-          <t>The missing number: how far the leg swings outward from centerline during a stride to clear the locked knee.</t>
+          <t>Angle needed to complete the reach-behind-head task, not a full ROM max. Not applied as a joint limit.</t>
         </is>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>NEEDED: not yet sourced (target: gait-lab / Journal of Prosthetics &amp; Orthotics studies of KAFO users)</t>
-        </is>
-      </c>
-      <c r="P30" s="5" t="inlineStr">
-        <is>
-          <t>placeholder</t>
-        </is>
-      </c>
-      <c r="Q30" s="5" t="inlineStr">
-        <is>
-          <t>n/a: functional measure, not a joint angle</t>
+          <t>PMC11115294 (hemiplegia reach-behind-head study)</t>
+        </is>
+      </c>
+      <c r="P30" s="3" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="Q30" s="3" t="inlineStr">
+        <is>
+          <t>Elbow flexion, +α about humerus Z; Z-X-Y; Wu et al. 2005 (ISB Part II) 3.4.1</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>arthritis-shoulder-flex</t>
+          <t>kafo-knee-flex-locked</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>shoulder_affected</t>
+          <t>knee_affected</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>trunk</t>
+          <t>hip_affected</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -2794,104 +2802,120 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>arthritis (RA or OA)</t>
+          <t>KAFO (locked)</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>moderate/severe</t>
-        </is>
-      </c>
-      <c r="G31" s="2" t="n"/>
-      <c r="H31" s="2" t="n"/>
+          <t>typical</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
           <t>joint_limits</t>
         </is>
       </c>
-      <c r="J31" s="2" t="n"/>
-      <c r="K31" s="2" t="n"/>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>n/a (mechanically fixed)</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>fixed</t>
+        </is>
+      </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>either or both sides</t>
-        </is>
-      </c>
-      <c r="M31" s="2" t="n"/>
+          <t>affected side</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>requires circumduction or hip-hike to clear the leg</t>
+        </is>
+      </c>
       <c r="N31" s="2" t="inlineStr">
         <is>
-          <t>Reach reduction not yet sourced. Needs per-joint goniometry or functional reach test (FRT) data on arthritis populations.</t>
+          <t>Leg cannot bend. Wearer compensates via circumduction (lateral hip swing) or hip-hike, which this row does not capture.</t>
         </is>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
-          <t>NEEDED: not yet sourced</t>
-        </is>
-      </c>
-      <c r="P31" s="5" t="inlineStr">
-        <is>
-          <t>placeholder</t>
-        </is>
-      </c>
-      <c r="Q31" s="5" t="inlineStr">
-        <is>
-          <t>Thoracohumeral elevation in plane of elevation 90° (forward); Y-X-Y; Wu et al. 2005 (ISB Part II) 2.4.7</t>
+          <t>General orthotics principle (KAFO knee joint typically locked near full extension); not a specific citation</t>
+        </is>
+      </c>
+      <c r="P31" s="4" t="inlineStr">
+        <is>
+          <t>interpolated</t>
+        </is>
+      </c>
+      <c r="Q31" s="4" t="inlineStr">
+        <is>
+          <t>Knee flexion; Grood &amp; Suntay 1983 (the knee convention ISB uses)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>arthritis-shoulder-abd</t>
+          <t>kafo-knee-circumduction</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>shoulder_affected</t>
+          <t>knee_affected</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>trunk</t>
+          <t>hip_affected</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>abduction</t>
+          <t>lateral sweep (circumduction)</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>arthritis (RA or OA)</t>
+          <t>KAFO (locked)</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>moderate/severe</t>
+          <t>typical</t>
         </is>
       </c>
       <c r="G32" s="2" t="n"/>
       <c r="H32" s="2" t="n"/>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>joint_limits</t>
+          <t>sweep_width</t>
         </is>
       </c>
       <c r="J32" s="2" t="n"/>
       <c r="K32" s="2" t="n"/>
       <c r="L32" s="2" t="inlineStr">
         <is>
-          <t>either or both sides</t>
+          <t>affected side</t>
         </is>
       </c>
       <c r="M32" s="2" t="n"/>
       <c r="N32" s="2" t="inlineStr">
         <is>
-          <t>Split from the original 'flexion/abduction' row so each axis has its own row.</t>
+          <t>The missing number: how far the leg swings outward from centerline during a stride to clear the locked knee.</t>
         </is>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>NEEDED: not yet sourced</t>
+          <t>NEEDED: not yet sourced (target: gait-lab / Journal of Prosthetics &amp; Orthotics studies of KAFO users)</t>
         </is>
       </c>
       <c r="P32" s="5" t="inlineStr">
@@ -2901,24 +2925,24 @@
       </c>
       <c r="Q32" s="5" t="inlineStr">
         <is>
-          <t>Thoracohumeral elevation in plane of elevation 0° (sideways); Y-X-Y; Wu et al. 2005 (ISB Part II) 2.4.7</t>
+          <t>n/a: functional measure, not a joint angle</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>arthritis-hip-flex</t>
+          <t>arthritis-shoulder-flex</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>hip_affected</t>
+          <t>shoulder_affected</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>pelvis</t>
+          <t>trunk</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -2953,7 +2977,7 @@
       <c r="M33" s="2" t="n"/>
       <c r="N33" s="2" t="inlineStr">
         <is>
-          <t>Reach reduction not yet sourced.</t>
+          <t>Reach reduction not yet sourced. Needs per-joint goniometry or functional reach test (FRT) data on arthritis populations.</t>
         </is>
       </c>
       <c r="O33" s="2" t="inlineStr">
@@ -2968,29 +2992,29 @@
       </c>
       <c r="Q33" s="5" t="inlineStr">
         <is>
-          <t>Hip flexion, +α about pelvis Z; Wu et al. 2002 (ISB Part I)</t>
+          <t>Thoracohumeral elevation in plane of elevation 90° (forward); Y-X-Y; Wu et al. 2005 (ISB Part II) 2.4.7</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>arthritis-knee-flex</t>
+          <t>arthritis-shoulder-abd</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>knee_affected</t>
+          <t>shoulder_affected</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>hip_affected</t>
+          <t>trunk</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>flexion</t>
+          <t>abduction</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -3020,7 +3044,7 @@
       <c r="M34" s="2" t="n"/>
       <c r="N34" s="2" t="inlineStr">
         <is>
-          <t>Reach/kneel reduction not yet sourced.</t>
+          <t>Split from the original 'flexion/abduction' row so each axis has its own row.</t>
         </is>
       </c>
       <c r="O34" s="2" t="inlineStr">
@@ -3035,29 +3059,29 @@
       </c>
       <c r="Q34" s="5" t="inlineStr">
         <is>
-          <t>Knee flexion; Grood &amp; Suntay 1983 (the knee convention ISB uses)</t>
+          <t>Thoracohumeral elevation in plane of elevation 0° (sideways); Y-X-Y; Wu et al. 2005 (ISB Part II) 2.4.7</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>arthritis-hand-grip</t>
+          <t>arthritis-hip-flex</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>hand_affected</t>
+          <t>hip_affected</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>wrist_affected</t>
+          <t>pelvis</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>grip / finger flexion</t>
+          <t>flexion</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
@@ -3087,7 +3111,7 @@
       <c r="M35" s="2" t="n"/>
       <c r="N35" s="2" t="inlineStr">
         <is>
-          <t>Grip strength reduction not yet sourced. Relevant once a hand card is built.</t>
+          <t>Reach reduction not yet sourced.</t>
         </is>
       </c>
       <c r="O35" s="2" t="inlineStr">
@@ -3102,59 +3126,59 @@
       </c>
       <c r="Q35" s="5" t="inlineStr">
         <is>
-          <t>MCP/IP flexion, +α about proximal segment Z; Wu et al. 2005 (ISB Part II) 4.4.1</t>
+          <t>Hip flexion, +α about pelvis Z; Wu et al. 2002 (ISB Part I)</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>neglect-reach-shift</t>
+          <t>arthritis-knee-flex</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>shoulder_affected</t>
+          <t>knee_affected</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>trunk</t>
+          <t>hip_affected</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>spatial reach-envelope shift</t>
+          <t>flexion</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>hemiplegia (neglect)</t>
+          <t>arthritis (RA or OA)</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>typical</t>
+          <t>moderate/severe</t>
         </is>
       </c>
       <c r="G36" s="2" t="n"/>
       <c r="H36" s="2" t="n"/>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>envelope_shift</t>
+          <t>joint_limits</t>
         </is>
       </c>
       <c r="J36" s="2" t="n"/>
       <c r="K36" s="2" t="n"/>
       <c r="L36" s="2" t="inlineStr">
         <is>
-          <t>affected side</t>
+          <t>either or both sides</t>
         </is>
       </c>
       <c r="M36" s="2" t="n"/>
       <c r="N36" s="2" t="inlineStr">
         <is>
-          <t>Neglect-cone angle: how far the reach envelope shifts/shrinks toward the unaffected side.</t>
+          <t>Reach/kneel reduction not yet sourced.</t>
         </is>
       </c>
       <c r="O36" s="2" t="inlineStr">
@@ -3169,14 +3193,14 @@
       </c>
       <c r="Q36" s="5" t="inlineStr">
         <is>
-          <t>n/a: functional measure, not a joint angle</t>
+          <t>Knee flexion; Grood &amp; Suntay 1983 (the knee convention ISB uses)</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>crutch-wet-reach</t>
+          <t>arthritis-hand-grip</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -3191,24 +3215,24 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>functional reach</t>
+          <t>grip / finger flexion</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>crutch-assisted, wet floor</t>
+          <t>arthritis (RA or OA)</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>typical</t>
+          <t>moderate/severe</t>
         </is>
       </c>
       <c r="G37" s="2" t="n"/>
       <c r="H37" s="2" t="n"/>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>reach_reduction</t>
+          <t>joint_limits</t>
         </is>
       </c>
       <c r="J37" s="2" t="n"/>
@@ -3218,27 +3242,161 @@
           <t>either or both sides</t>
         </is>
       </c>
-      <c r="M37" s="2" t="inlineStr">
+      <c r="M37" s="2" t="n"/>
+      <c r="N37" s="2" t="inlineStr">
+        <is>
+          <t>Grip strength reduction not yet sourced. Relevant once a hand card is built.</t>
+        </is>
+      </c>
+      <c r="O37" s="2" t="inlineStr">
+        <is>
+          <t>NEEDED: not yet sourced</t>
+        </is>
+      </c>
+      <c r="P37" s="5" t="inlineStr">
+        <is>
+          <t>placeholder</t>
+        </is>
+      </c>
+      <c r="Q37" s="5" t="inlineStr">
+        <is>
+          <t>MCP/IP flexion, +α about proximal segment Z; Wu et al. 2005 (ISB Part II) 4.4.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>neglect-reach-shift</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>shoulder_affected</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>trunk</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>spatial reach-envelope shift</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>hemiplegia (neglect)</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>typical</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="n"/>
+      <c r="H38" s="2" t="n"/>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>envelope_shift</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="n"/>
+      <c r="K38" s="2" t="n"/>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>affected side</t>
+        </is>
+      </c>
+      <c r="M38" s="2" t="n"/>
+      <c r="N38" s="2" t="inlineStr">
+        <is>
+          <t>Neglect-cone angle: how far the reach envelope shifts/shrinks toward the unaffected side.</t>
+        </is>
+      </c>
+      <c r="O38" s="2" t="inlineStr">
+        <is>
+          <t>NEEDED: not yet sourced</t>
+        </is>
+      </c>
+      <c r="P38" s="5" t="inlineStr">
+        <is>
+          <t>placeholder</t>
+        </is>
+      </c>
+      <c r="Q38" s="5" t="inlineStr">
+        <is>
+          <t>n/a: functional measure, not a joint angle</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>crutch-wet-reach</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>hand_affected</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>wrist_affected</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>functional reach</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>crutch-assisted, wet floor</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>typical</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="n"/>
+      <c r="H39" s="2" t="n"/>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>reach_reduction</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="n"/>
+      <c r="K39" s="2" t="n"/>
+      <c r="L39" s="2" t="inlineStr">
+        <is>
+          <t>either or both sides</t>
+        </is>
+      </c>
+      <c r="M39" s="2" t="inlineStr">
         <is>
           <t>requires free hand for balance</t>
         </is>
       </c>
-      <c r="N37" s="2" t="inlineStr">
+      <c r="N39" s="2" t="inlineStr">
         <is>
           <t>Reach reduction on a compromised-traction surface, not yet sourced.</t>
         </is>
       </c>
-      <c r="O37" s="2" t="inlineStr">
+      <c r="O39" s="2" t="inlineStr">
         <is>
           <t>NEEDED: not yet sourced</t>
         </is>
       </c>
-      <c r="P37" s="5" t="inlineStr">
+      <c r="P39" s="5" t="inlineStr">
         <is>
           <t>placeholder</t>
         </is>
       </c>
-      <c r="Q37" s="5" t="inlineStr">
+      <c r="Q39" s="5" t="inlineStr">
         <is>
           <t>n/a: functional measure, not a joint angle</t>
         </is>
@@ -4037,7 +4195,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>How the verifier uses the numbers. joint_limits: the joint can move from 0 to ROM_max. score_band: a clinical scoring band; the verifier uses the band's lower edge so the design has to work for everyone in the band. task_threshold: the angle a task needed; reported, never applied as a limit. sweep_width / envelope_shift / reach_reduction: functional measures, not yet used by the verifier.</t>
+          <t>How the verifier uses the numbers. joint_limits: the joint can move from 0 to ROM_max. score_band: a band of values (a clinical scoring band, or a study's mean ± 1 standard deviation); the verifier uses the band's lower edge so the design has to work for everyone in the band. task_threshold: the angle a task needed; reported, never applied as a limit. sweep_width / envelope_shift / reach_reduction: functional measures, not yet used by the verifier.</t>
         </is>
       </c>
     </row>
@@ -4261,7 +4419,6 @@
         </is>
       </c>
     </row>
-    <row r="31"/>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
@@ -4285,7 +4442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -4396,6 +4553,13 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Added two stroke active arm-lift (shoulder flexion) cards from Taketomi 2023 and Yim &amp; Kim 2024, as bands of mean ± 1 SD. Not used by any profile yet.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fill arthritis shoulder and knee flexion cards (end-stage OA)
Shoulder forward elevation 96 ± 30 (Jensen 2021, n=377, ages 70+, before
shoulder replacement) and knee flexion 114.3 ± 13.4 (Lee 2025, worst KL-4
subgroup), stored as mean ± 1 SD bands; the verifier uses the lower edge.
Shoulder abduction and hand grip stay placeholders (no published degrees);
hip waits for checking. Tests that used these as example placeholders now
use the abduction and hip cards.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UEvCJX2bMQCcooJE7fGgnQ
</commit_message>
<xml_diff>
--- a/data/card_library.xlsx
+++ b/data/card_library.xlsx
@@ -2952,22 +2952,30 @@
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>arthritis (RA or OA)</t>
+          <t>arthritis (osteoarthritis)</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>moderate/severe</t>
-        </is>
-      </c>
-      <c r="G33" s="2" t="n"/>
-      <c r="H33" s="2" t="n"/>
+          <t>end-stage (before shoulder replacement)</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="n">
+        <v>66</v>
+      </c>
+      <c r="H33" s="2" t="n">
+        <v>126</v>
+      </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>joint_limits</t>
-        </is>
-      </c>
-      <c r="J33" s="2" t="n"/>
+          <t>score_band</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>reduced</t>
+        </is>
+      </c>
       <c r="K33" s="2" t="n"/>
       <c r="L33" s="2" t="inlineStr">
         <is>
@@ -2977,17 +2985,17 @@
       <c r="M33" s="2" t="n"/>
       <c r="N33" s="2" t="inlineStr">
         <is>
-          <t>Reach reduction not yet sourced. Needs per-joint goniometry or functional reach test (FRT) data on arthritis populations.</t>
+          <t>Forward elevation (arm lifted forward), mean 96 ± 1 SD 30 degrees; external rotation 26 ± 20. 377 shoulders, ages 70+, measured just before anatomic shoulder replacement. Verifier uses the lower edge. End-stage only: no published degrees for early shoulder OA.</t>
         </is>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
-          <t>NEEDED: not yet sourced</t>
+          <t>Jensen et al. 2021, J Shoulder Elbow Surg 30(7S):S131-S139, doi:10.1016/j.jse.2020.11.030 (PMID 33484829), preoperative values</t>
         </is>
       </c>
       <c r="P33" s="5" t="inlineStr">
         <is>
-          <t>placeholder</t>
+          <t>sourced</t>
         </is>
       </c>
       <c r="Q33" s="5" t="inlineStr">
@@ -3153,22 +3161,30 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>arthritis (RA or OA)</t>
+          <t>arthritis (osteoarthritis)</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>moderate/severe</t>
-        </is>
-      </c>
-      <c r="G36" s="2" t="n"/>
-      <c r="H36" s="2" t="n"/>
+          <t>end-stage (KL grade 4, worst subgroup)</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="n">
+        <v>100.9</v>
+      </c>
+      <c r="H36" s="2" t="n">
+        <v>127.7</v>
+      </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>joint_limits</t>
-        </is>
-      </c>
-      <c r="J36" s="2" t="n"/>
+          <t>score_band</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>reduced</t>
+        </is>
+      </c>
       <c r="K36" s="2" t="n"/>
       <c r="L36" s="2" t="inlineStr">
         <is>
@@ -3178,17 +3194,17 @@
       <c r="M36" s="2" t="n"/>
       <c r="N36" s="2" t="inlineStr">
         <is>
-          <t>Reach/kneel reduction not yet sourced.</t>
+          <t>Full knee flexion 114.3 ± 1 SD 13.4 degrees in the worst of three KL-4 subgroups (joint space lost in both views); another subgroup averaged 121.2. Chosen as the cautious case. 300 patients, average age about 72. Verifier uses the lower edge.</t>
         </is>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
-          <t>NEEDED: not yet sourced</t>
+          <t>Lee et al. 2025, BMC Musculoskelet Disord 26:696, doi:10.1186/s12891-025-08943-y (PMID 40696346), group 1</t>
         </is>
       </c>
       <c r="P36" s="5" t="inlineStr">
         <is>
-          <t>placeholder</t>
+          <t>sourced</t>
         </is>
       </c>
       <c r="Q36" s="5" t="inlineStr">
@@ -4442,7 +4458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -4560,6 +4576,13 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Filled two arthritis cards (Oct 8): shoulder flexion 66-126 (Jensen 2021) and knee flexion 100.9-127.7 (Lee 2025), both end-stage osteoarthritis, as mean ± 1 SD bands. Shoulder abduction and hand grip stay gaps (no published degrees); hip waits for checking.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Correct wheelchair above-shoulder cap to IDeA's 41 of 276 (about 15%)
The ~21% figure had no source; IDeA Design Resource #20, Note 1 says 235 of
276 manual wheelchair users could grasp and reach above shoulder height. The
cap is only a fallback when data/idea_reach.json is missing.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UEvCJX2bMQCcooJE7fGgnQ
</commit_message>
<xml_diff>
--- a/data/card_library.xlsx
+++ b/data/card_library.xlsx
@@ -3871,16 +3871,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0.21</v>
+        <v>0.15</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>~21% of wheelchair users cannot reach above shoulder height. Applied as a population-level caution, not a per-person ROM limit.</t>
+          <t>41 of the 276 manual wheelchair users recruited (about 15%) could not grasp and reach above shoulder height, so they were not measured. Applied as a population-level caution, not a per-person ROM limit. Used only when data/idea_reach.json is missing; otherwise the full IDeA charts are used. (Corrected Oct 8, 2026 from an unsourced ~21%.)</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>IDeA Center / University at Buffalo, U.S. Access Board-funded anthropometry study</t>
+          <t>IDeA Center, University at Buffalo (U.S. Access Board-funded). D'Souza, Steinfeld, Paquet, Feathers. Design Resource #20: Functional Reach Capability for Wheeled Mobility Users, Jan 4, 2011, Note 1. https://idea.ap.buffalo.edu/wp-content/uploads/sites/110/2019/08/20.pdf</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -4458,7 +4458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A17"/>
+  <dimension ref="A1:A18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -4583,6 +4583,13 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Oct 8, 2026: wheelchair-above-shoulder cap corrected from ~21% (no source found) to 41 of 276, about 15%, per IDeA Design Resource #20, Note 1.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>